<commit_message>
Ask about marital status, real estate, and other assets before building a plan
</commit_message>
<xml_diff>
--- a/skills/retirement-cash-flow-planner/assets/retirement-plan-template.xlsx
+++ b/skills/retirement-cash-flow-planner/assets/retirement-plan-template.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="170">
   <si>
     <t xml:space="preserve">PERSONAL RETIREMENT FINANCIAL PLAN</t>
   </si>
@@ -533,6 +533,9 @@
   </si>
   <si>
     <t xml:space="preserve">Real Estate Equity (enter manually or link to a Properties tab)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other Assets (gold, pension, business interest, etc. — if any)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL NET WORTH</t>
@@ -689,7 +692,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -742,10 +745,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -756,6 +755,14 @@
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1919,43 +1926,43 @@
       <c r="A7" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="7" t="n">
         <f aca="false">IF(B$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,B$2-Assumptions!$B$17),0)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="7" t="n">
         <f aca="false">IF(C$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,C$2-Assumptions!$B$17),0)</f>
         <v>0</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="7" t="n">
         <f aca="false">IF(D$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,D$2-Assumptions!$B$17),0)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="7" t="n">
         <f aca="false">IF(E$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,E$2-Assumptions!$B$17),0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="7" t="n">
         <f aca="false">IF(F$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,F$2-Assumptions!$B$17),0)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="7" t="n">
         <f aca="false">IF(G$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,G$2-Assumptions!$B$17),0)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="13" t="n">
+      <c r="H7" s="7" t="n">
         <f aca="false">IF(H$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,H$2-Assumptions!$B$17),0)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="I7" s="7" t="n">
         <f aca="false">IF(I$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,I$2-Assumptions!$B$17),0)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="7" t="n">
         <f aca="false">IF(J$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,J$2-Assumptions!$B$17),0)</f>
         <v>30000</v>
       </c>
-      <c r="K7" s="13" t="n">
+      <c r="K7" s="7" t="n">
         <f aca="false">IF(K$2&gt;=Assumptions!$B$17,Assumptions!$E$27*(1+Assumptions!$E$28)^MAX(0,K$2-Assumptions!$B$17),0)</f>
         <v>30750</v>
       </c>
@@ -1964,43 +1971,43 @@
       <c r="A8" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="7" t="n">
         <f aca="false">IF(B$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,B$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="7" t="n">
         <f aca="false">IF(C$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,C$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="7" t="n">
         <f aca="false">IF(D$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,D$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="7" t="n">
         <f aca="false">IF(E$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,E$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="7" t="n">
         <f aca="false">IF(F$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,F$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="G8" s="7" t="n">
         <f aca="false">IF(G$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,G$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="13" t="n">
+      <c r="H8" s="7" t="n">
         <f aca="false">IF(H$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,H$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="13" t="n">
+      <c r="I8" s="7" t="n">
         <f aca="false">IF(I$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,I$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="J8" s="13" t="n">
+      <c r="J8" s="7" t="n">
         <f aca="false">IF(J$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,J$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
-      <c r="K8" s="13" t="n">
+      <c r="K8" s="7" t="n">
         <f aca="false">IF(K$2&gt;=Assumptions!$B$18,Assumptions!$E$26*(1+Assumptions!$E$28)^MAX(0,K$2-Assumptions!$B$18),0)</f>
         <v>0</v>
       </c>
@@ -2009,43 +2016,43 @@
       <c r="A9" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="13" t="n">
         <f aca="false">SUM(B5:B8)</f>
         <v>36000</v>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="13" t="n">
         <f aca="false">SUM(C5:C8)</f>
         <v>37080</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="13" t="n">
         <f aca="false">SUM(D5:D8)</f>
         <v>38192.4</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="13" t="n">
         <f aca="false">SUM(E5:E8)</f>
         <v>39338.172</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="13" t="n">
         <f aca="false">SUM(F5:F8)</f>
         <v>40518.31716</v>
       </c>
-      <c r="G9" s="14" t="n">
+      <c r="G9" s="13" t="n">
         <f aca="false">SUM(G5:G8)</f>
         <v>41733.8666748</v>
       </c>
-      <c r="H9" s="14" t="n">
+      <c r="H9" s="13" t="n">
         <f aca="false">SUM(H5:H8)</f>
         <v>42985.882675044</v>
       </c>
-      <c r="I9" s="14" t="n">
+      <c r="I9" s="13" t="n">
         <f aca="false">SUM(I5:I8)</f>
         <v>44275.4591552953</v>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="13" t="n">
         <f aca="false">SUM(J5:J8)</f>
         <v>75603.7229299542</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="K9" s="13" t="n">
         <f aca="false">SUM(K5:K8)</f>
         <v>77721.8346178528</v>
       </c>
@@ -2159,43 +2166,43 @@
       <c r="A14" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="13" t="n">
         <f aca="false">SUM(B12:B13)</f>
         <v>-117600</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="13" t="n">
         <f aca="false">SUM(C12:C13)</f>
         <v>-121560</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="13" t="n">
         <f aca="false">SUM(D12:D13)</f>
         <v>-125660.4</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="13" t="n">
         <f aca="false">SUM(E12:E13)</f>
         <v>-129906.492</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="13" t="n">
         <f aca="false">SUM(F12:F13)</f>
         <v>-134303.78076</v>
       </c>
-      <c r="G14" s="14" t="n">
+      <c r="G14" s="13" t="n">
         <f aca="false">SUM(G12:G13)</f>
         <v>-138857.9928828</v>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="H14" s="13" t="n">
         <f aca="false">SUM(H12:H13)</f>
         <v>-143575.086304284</v>
       </c>
-      <c r="I14" s="14" t="n">
+      <c r="I14" s="13" t="n">
         <f aca="false">SUM(I12:I13)</f>
         <v>-148461.260210163</v>
       </c>
-      <c r="J14" s="14" t="n">
+      <c r="J14" s="13" t="n">
         <f aca="false">SUM(J12:J13)</f>
         <v>-153522.965399055</v>
       </c>
-      <c r="K14" s="14" t="n">
+      <c r="K14" s="13" t="n">
         <f aca="false">SUM(K12:K13)</f>
         <v>-158766.915112743</v>
       </c>
@@ -2558,43 +2565,43 @@
       <c r="A6" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="13" t="n">
         <f aca="false">MAX(0,B4+B5)</f>
         <v>108948</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="13" t="n">
         <f aca="false">MAX(0,C4+C5)</f>
         <v>113714.4</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="13" t="n">
         <f aca="false">MAX(0,D4+D5)</f>
         <v>118651.44</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="13" t="n">
         <f aca="false">MAX(0,E4+E5)</f>
         <v>123765.6216</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="13" t="n">
         <f aca="false">MAX(0,F4+F5)</f>
         <v>129063.710568</v>
       </c>
-      <c r="G6" s="14" t="n">
+      <c r="G6" s="13" t="n">
         <f aca="false">MAX(0,G4+G5)</f>
         <v>134552.74822104</v>
       </c>
-      <c r="H6" s="14" t="n">
+      <c r="H6" s="13" t="n">
         <f aca="false">MAX(0,H4+H5)</f>
         <v>140240.063320471</v>
       </c>
-      <c r="I6" s="14" t="n">
+      <c r="I6" s="13" t="n">
         <f aca="false">MAX(0,I4+I5)</f>
         <v>146133.284505525</v>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="13" t="n">
         <f aca="false">MAX(0,J4+J5)</f>
         <v>143840.353290403</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="K6" s="13" t="n">
         <f aca="false">MAX(0,K4+K5)</f>
         <v>149959.537651313</v>
       </c>
@@ -2648,43 +2655,43 @@
       <c r="A9" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="14" t="n">
         <f aca="false">IFERROR(B8/B6,0)</f>
         <v>0.126634357675221</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="14" t="n">
         <f aca="false">IFERROR(C8/C6,0)</f>
         <v>0.130547828595147</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="14" t="n">
         <f aca="false">IFERROR(D8/D6,0)</f>
         <v>0.134269898452138</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="14" t="n">
         <f aca="false">IFERROR(E8/E6,0)</f>
         <v>0.137812395166769</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="14" t="n">
         <f aca="false">IFERROR(F8/F6,0)</f>
         <v>0.141186211404943</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="14" t="n">
         <f aca="false">IFERROR(G8/G6,0)</f>
         <v>0.144401395478822</v>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H9" s="14" t="n">
         <f aca="false">IFERROR(H8/H6,0)</f>
         <v>0.147467231836916</v>
       </c>
-      <c r="I9" s="15" t="n">
+      <c r="I9" s="14" t="n">
         <f aca="false">IFERROR(I8/I6,0)</f>
         <v>0.150392312508275</v>
       </c>
-      <c r="J9" s="15" t="n">
+      <c r="J9" s="14" t="n">
         <f aca="false">IFERROR(J8/J6,0)</f>
         <v>0.149282709842463</v>
       </c>
-      <c r="K9" s="15" t="n">
+      <c r="K9" s="14" t="n">
         <f aca="false">IFERROR(K8/K6,0)</f>
         <v>0.152168369152671</v>
       </c>
@@ -2783,43 +2790,43 @@
       <c r="A15" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="13" t="n">
         <f aca="false">B8+B11+B13</f>
         <v>19522.48</v>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="13" t="n">
         <f aca="false">C8+C11+C13</f>
         <v>20907.8512</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="13" t="n">
         <f aca="false">D8+D11+D13</f>
         <v>22495.41592</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="13" t="n">
         <f aca="false">E8+E11+E13</f>
         <v>24139.6940968</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="13" t="n">
         <f aca="false">F8+F11+F13</f>
         <v>25842.841459864</v>
       </c>
-      <c r="G15" s="14" t="n">
+      <c r="G15" s="13" t="n">
         <f aca="false">G8+G11+G13</f>
         <v>27607.1011268279</v>
       </c>
-      <c r="H15" s="14" t="n">
+      <c r="H15" s="13" t="n">
         <f aca="false">H8+H11+H13</f>
         <v>29434.8073609592</v>
       </c>
-      <c r="I15" s="14" t="n">
+      <c r="I15" s="13" t="n">
         <f aca="false">I8+I11+I13</f>
         <v>31328.3894981307</v>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="13" t="n">
         <f aca="false">J8+J11+J13</f>
         <v>30661.1760512344</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="K15" s="13" t="n">
         <f aca="false">K8+K11+K13</f>
         <v>32628.4690003393</v>
       </c>
@@ -2828,43 +2835,43 @@
       <c r="A16" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="14" t="n">
         <f aca="false">IFERROR(B15/B4,0)</f>
         <v>0.139001480975165</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="14" t="n">
         <f aca="false">IFERROR(C15/C4,0)</f>
         <v>0.143979186637138</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="14" t="n">
         <f aca="false">IFERROR(D15/D4,0)</f>
         <v>0.149818183029081</v>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E16" s="14" t="n">
         <f aca="false">IFERROR(E15/E4,0)</f>
         <v>0.15547352883428</v>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="14" t="n">
         <f aca="false">IFERROR(F15/F4,0)</f>
         <v>0.160950699061725</v>
       </c>
-      <c r="G16" s="15" t="n">
+      <c r="G16" s="14" t="n">
         <f aca="false">IFERROR(G15/G4,0)</f>
         <v>0.166255008860672</v>
       </c>
-      <c r="H16" s="15" t="n">
+      <c r="H16" s="14" t="n">
         <f aca="false">IFERROR(H15/H4,0)</f>
         <v>0.171391618192391</v>
       </c>
-      <c r="I16" s="15" t="n">
+      <c r="I16" s="14" t="n">
         <f aca="false">IFERROR(I15/I4,0)</f>
         <v>0.176365536365209</v>
       </c>
-      <c r="J16" s="15" t="n">
+      <c r="J16" s="14" t="n">
         <f aca="false">IFERROR(J15/J4,0)</f>
         <v>0.174866626397476</v>
       </c>
-      <c r="K16" s="15" t="n">
+      <c r="K16" s="14" t="n">
         <f aca="false">IFERROR(K15/K4,0)</f>
         <v>0.179811264939059</v>
       </c>
@@ -2873,43 +2880,43 @@
       <c r="A18" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="B18" s="14" t="n">
+      <c r="B18" s="13" t="n">
         <f aca="false">B4-B15</f>
         <v>120925.52</v>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="13" t="n">
         <f aca="false">C4-C15</f>
         <v>124306.5488</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="13" t="n">
         <f aca="false">D4-D15</f>
         <v>127656.02408</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E18" s="13" t="n">
         <f aca="false">E4-E15</f>
         <v>131125.9275032</v>
       </c>
-      <c r="F18" s="14" t="n">
+      <c r="F18" s="13" t="n">
         <f aca="false">F4-F15</f>
         <v>134720.869108136</v>
       </c>
-      <c r="G18" s="14" t="n">
+      <c r="G18" s="13" t="n">
         <f aca="false">G4-G15</f>
         <v>138445.647094212</v>
       </c>
-      <c r="H18" s="14" t="n">
+      <c r="H18" s="13" t="n">
         <f aca="false">H4-H15</f>
         <v>142305.255959512</v>
       </c>
-      <c r="I18" s="14" t="n">
+      <c r="I18" s="13" t="n">
         <f aca="false">I4-I15</f>
         <v>146304.895007395</v>
       </c>
-      <c r="J18" s="14" t="n">
+      <c r="J18" s="13" t="n">
         <f aca="false">J4-J15</f>
         <v>144679.177239169</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="K18" s="13" t="n">
         <f aca="false">K4-K15</f>
         <v>148831.068650974</v>
       </c>
@@ -2957,19 +2964,19 @@
       <c r="A2" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="15" t="s">
         <v>152</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="15" t="s">
         <v>155</v>
       </c>
       <c r="G2" s="9" t="s">
@@ -3322,7 +3329,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="55"/>
@@ -3639,48 +3646,84 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B11" s="14" t="n">
-        <f aca="false">SUM(B4:B9)</f>
+      <c r="B10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="B12" s="17" t="n">
+        <f aca="false">SUM(B4:B10)</f>
         <v>1970000</v>
       </c>
-      <c r="C11" s="14" t="n">
-        <f aca="false">SUM(C4:C9)</f>
+      <c r="C12" s="17" t="n">
+        <f aca="false">SUM(C4:C10)</f>
         <v>1872752</v>
       </c>
-      <c r="D11" s="14" t="n">
-        <f aca="false">SUM(D4:D9)</f>
+      <c r="D12" s="17" t="n">
+        <f aca="false">SUM(D4:D10)</f>
         <v>1772129.6</v>
       </c>
-      <c r="E11" s="14" t="n">
-        <f aca="false">SUM(E4:E9)</f>
+      <c r="E12" s="17" t="n">
+        <f aca="false">SUM(E4:E10)</f>
         <v>1668008.48</v>
       </c>
-      <c r="F11" s="14" t="n">
-        <f aca="false">SUM(F4:F9)</f>
+      <c r="F12" s="17" t="n">
+        <f aca="false">SUM(F4:F10)</f>
         <v>1560259.4336</v>
       </c>
-      <c r="G11" s="14" t="n">
-        <f aca="false">SUM(G4:G9)</f>
+      <c r="G12" s="17" t="n">
+        <f aca="false">SUM(G4:G10)</f>
         <v>1448748.163904</v>
       </c>
-      <c r="H11" s="14" t="n">
-        <f aca="false">SUM(H4:H9)</f>
+      <c r="H12" s="17" t="n">
+        <f aca="false">SUM(H4:H10)</f>
         <v>1333335.07046528</v>
       </c>
-      <c r="I11" s="14" t="n">
-        <f aca="false">SUM(I4:I9)</f>
+      <c r="I12" s="17" t="n">
+        <f aca="false">SUM(I4:I10)</f>
         <v>1213875.02686554</v>
       </c>
-      <c r="J11" s="14" t="n">
-        <f aca="false">SUM(J4:J9)</f>
+      <c r="J12" s="17" t="n">
+        <f aca="false">SUM(J4:J10)</f>
         <v>1090217.14850151</v>
       </c>
-      <c r="K11" s="14" t="n">
-        <f aca="false">SUM(K4:K9)</f>
+      <c r="K12" s="17" t="n">
+        <f aca="false">SUM(K4:K10)</f>
         <v>1147286.35104328</v>
       </c>
     </row>

</xml_diff>